<commit_message>
feat(ai): prompt ile tabaktaki yemeği tanıma, çatal bıçak var ise ölçek referansı olarak kullansın, tahmin olarak işaretleniyor, kullanıcı onayı ile dbye gidiyor
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BFF644-F1E8-4E82-824F-F85C1CCD9464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB54609-98C3-41C5-908F-6886EA15291E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ozet Dashboard" sheetId="1" r:id="rId1"/>
@@ -2460,10 +2460,13 @@
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -2471,16 +2474,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2894,7 +2894,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="29"/>
@@ -2904,7 +2904,7 @@
       <c r="F1" s="29"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="29"/>
@@ -2922,181 +2922,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3137,11 +3137,11 @@
       </c>
       <c r="D23" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$64,'Sprint Plani'!$A$4:$A$64,$A23,'Sprint Plani'!$K$4:$K$64,"Tamamlandı")</f>
-        <v>9</v>
+        <v>16.5</v>
       </c>
       <c r="E23" s="7">
         <f>IFERROR($D23/$C23,0)</f>
-        <v>0.25</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>41</v>
@@ -3209,11 +3209,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>9</v>
+        <v>16.5</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>7.1428571428571425E-2</v>
+        <v>0.13095238095238096</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3498,7 +3498,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="34" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="29"/>
@@ -3508,7 +3508,7 @@
       <c r="F46" s="29"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="36" t="s">
+      <c r="A47" s="34" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="29"/>
@@ -3518,7 +3518,7 @@
       <c r="F47" s="29"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="36" t="s">
+      <c r="A48" s="34" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="29"/>
@@ -3528,7 +3528,7 @@
       <c r="F48" s="29"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="36" t="s">
+      <c r="A49" s="34" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="29"/>
@@ -3538,7 +3538,7 @@
       <c r="F49" s="29"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="36" t="s">
+      <c r="A50" s="34" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="29"/>
@@ -3548,7 +3548,7 @@
       <c r="F50" s="29"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="36" t="s">
+      <c r="A51" s="34" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="29"/>
@@ -3558,7 +3558,7 @@
       <c r="F51" s="29"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="36" t="s">
+      <c r="A52" s="34" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="29"/>
@@ -3569,14 +3569,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3593,6 +3585,14 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3619,7 +3619,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>88</v>
       </c>
       <c r="B1" s="29"/>
@@ -3634,7 +3634,7 @@
       <c r="K1" s="29"/>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>89</v>
       </c>
       <c r="B2" s="29"/>
@@ -3855,7 +3855,7 @@
         <v>116</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -3890,7 +3890,7 @@
         <v>120</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3925,7 +3925,7 @@
         <v>125</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -5819,15 +5819,15 @@
       </c>
     </row>
     <row r="65" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="31" t="s">
+      <c r="A65" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="B65" s="32"/>
-      <c r="C65" s="32"/>
-      <c r="D65" s="32"/>
-      <c r="E65" s="32"/>
-      <c r="F65" s="32"/>
-      <c r="G65" s="32"/>
+      <c r="B65" s="33"/>
+      <c r="C65" s="33"/>
+      <c r="D65" s="33"/>
+      <c r="E65" s="33"/>
+      <c r="F65" s="33"/>
+      <c r="G65" s="33"/>
       <c r="H65" s="21">
         <f>SUM(H4:H64)</f>
         <v>126</v>
@@ -5840,7 +5840,7 @@
       <c r="K65" s="20"/>
     </row>
     <row r="67" spans="1:11" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="28" t="s">
+      <c r="A67" s="30" t="s">
         <v>379</v>
       </c>
       <c r="B67" s="29"/>
@@ -5855,7 +5855,7 @@
       <c r="K67" s="29"/>
     </row>
     <row r="68" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="28" t="s">
+      <c r="A68" s="30" t="s">
         <v>380</v>
       </c>
       <c r="B68" s="29"/>
@@ -5870,7 +5870,7 @@
       <c r="K68" s="29"/>
     </row>
     <row r="69" spans="1:11" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="28" t="s">
+      <c r="A69" s="30" t="s">
         <v>381</v>
       </c>
       <c r="B69" s="29"/>
@@ -5885,7 +5885,7 @@
       <c r="K69" s="29"/>
     </row>
     <row r="70" spans="1:11" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="28" t="s">
+      <c r="A70" s="30" t="s">
         <v>382</v>
       </c>
       <c r="B70" s="29"/>
@@ -5956,7 +5956,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>383</v>
       </c>
       <c r="B1" s="29"/>
@@ -5966,7 +5966,7 @@
       <c r="F1" s="29"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>384</v>
       </c>
       <c r="B2" s="29"/>
@@ -6582,7 +6582,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>481</v>
       </c>
       <c r="B1" s="29"/>
@@ -6593,7 +6593,7 @@
       <c r="G1" s="29"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>482</v>
       </c>
       <c r="B2" s="29"/>
@@ -7320,7 +7320,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>565</v>
       </c>
       <c r="B1" s="29"/>
@@ -7331,7 +7331,7 @@
       <c r="G1" s="29"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>566</v>
       </c>
       <c r="B2" s="29"/>
@@ -7699,7 +7699,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="34" t="s">
         <v>618</v>
       </c>
       <c r="B19" s="29"/>
@@ -7710,7 +7710,7 @@
       <c r="G19" s="29"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="34" t="s">
         <v>619</v>
       </c>
       <c r="B20" s="29"/>
@@ -7721,7 +7721,7 @@
       <c r="G20" s="29"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="34" t="s">
         <v>620</v>
       </c>
       <c r="B21" s="29"/>
@@ -7758,7 +7758,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>621</v>
       </c>
       <c r="B1" s="29"/>
@@ -7767,7 +7767,7 @@
       <c r="E1" s="29"/>
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>622</v>
       </c>
       <c r="B2" s="29"/>
@@ -8035,7 +8035,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>664</v>
       </c>
       <c r="B1" s="29"/>
@@ -8046,7 +8046,7 @@
       <c r="G1" s="29"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>665</v>
       </c>
       <c r="B2" s="29"/>

</xml_diff>

<commit_message>
feat(mobile):Flutter Projesi ve Katmanlı Mimari
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB54609-98C3-41C5-908F-6886EA15291E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A4D099-20F2-46B7-8E2B-90690C7CDEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ozet Dashboard" sheetId="1" r:id="rId1"/>
@@ -2474,13 +2474,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2922,181 +2922,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="36"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="36"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="36"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="36"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3137,11 +3137,11 @@
       </c>
       <c r="D23" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$64,'Sprint Plani'!$A$4:$A$64,$A23,'Sprint Plani'!$K$4:$K$64,"Tamamlandı")</f>
-        <v>16.5</v>
+        <v>27</v>
       </c>
       <c r="E23" s="7">
         <f>IFERROR($D23/$C23,0)</f>
-        <v>0.45833333333333331</v>
+        <v>0.75</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>41</v>
@@ -3209,11 +3209,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>16.5</v>
+        <v>27</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.13095238095238096</v>
+        <v>0.21428571428571427</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3498,7 +3498,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="34" t="s">
+      <c r="A46" s="36" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="29"/>
@@ -3508,7 +3508,7 @@
       <c r="F46" s="29"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="34" t="s">
+      <c r="A47" s="36" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="29"/>
@@ -3518,7 +3518,7 @@
       <c r="F47" s="29"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="34" t="s">
+      <c r="A48" s="36" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="29"/>
@@ -3528,7 +3528,7 @@
       <c r="F48" s="29"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="34" t="s">
+      <c r="A49" s="36" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="29"/>
@@ -3538,7 +3538,7 @@
       <c r="F49" s="29"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="34" t="s">
+      <c r="A50" s="36" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="29"/>
@@ -3548,7 +3548,7 @@
       <c r="F50" s="29"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="34" t="s">
+      <c r="A51" s="36" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="29"/>
@@ -3558,7 +3558,7 @@
       <c r="F51" s="29"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="34" t="s">
+      <c r="A52" s="36" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="29"/>
@@ -3569,6 +3569,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3585,14 +3593,6 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3960,7 +3960,7 @@
         <v>111</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -3995,7 +3995,7 @@
         <v>125</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -4030,7 +4030,7 @@
         <v>137</v>
       </c>
       <c r="K13" s="18" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4065,7 +4065,7 @@
         <v>105</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -4100,7 +4100,7 @@
         <v>99</v>
       </c>
       <c r="K15" s="18" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -7699,7 +7699,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="34" t="s">
+      <c r="A19" s="36" t="s">
         <v>618</v>
       </c>
       <c r="B19" s="29"/>
@@ -7710,7 +7710,7 @@
       <c r="G19" s="29"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="36" t="s">
         <v>619</v>
       </c>
       <c r="B20" s="29"/>
@@ -7721,7 +7721,7 @@
       <c r="G20" s="29"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
+      <c r="A21" s="36" t="s">
         <v>620</v>
       </c>
       <c r="B21" s="29"/>

</xml_diff>

<commit_message>
feat(mobile): 4 sekmeli navigason go_router ile yapıldı
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A4D099-20F2-46B7-8E2B-90690C7CDEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3109C570-949F-4F2F-BF88-140E86E3D8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ozet Dashboard" sheetId="1" r:id="rId1"/>
@@ -2474,13 +2474,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2922,181 +2922,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3137,11 +3137,11 @@
       </c>
       <c r="D23" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$64,'Sprint Plani'!$A$4:$A$64,$A23,'Sprint Plani'!$K$4:$K$64,"Tamamlandı")</f>
-        <v>27</v>
+        <v>32.5</v>
       </c>
       <c r="E23" s="7">
         <f>IFERROR($D23/$C23,0)</f>
-        <v>0.75</v>
+        <v>0.90277777777777779</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>41</v>
@@ -3209,11 +3209,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>27</v>
+        <v>32.5</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.21428571428571427</v>
+        <v>0.25793650793650796</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3498,7 +3498,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="34" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="29"/>
@@ -3508,7 +3508,7 @@
       <c r="F46" s="29"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="36" t="s">
+      <c r="A47" s="34" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="29"/>
@@ -3518,7 +3518,7 @@
       <c r="F47" s="29"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="36" t="s">
+      <c r="A48" s="34" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="29"/>
@@ -3528,7 +3528,7 @@
       <c r="F48" s="29"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="36" t="s">
+      <c r="A49" s="34" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="29"/>
@@ -3538,7 +3538,7 @@
       <c r="F49" s="29"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="36" t="s">
+      <c r="A50" s="34" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="29"/>
@@ -3548,7 +3548,7 @@
       <c r="F50" s="29"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="36" t="s">
+      <c r="A51" s="34" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="29"/>
@@ -3558,7 +3558,7 @@
       <c r="F51" s="29"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="36" t="s">
+      <c r="A52" s="34" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="29"/>
@@ -3569,14 +3569,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3593,6 +3585,14 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4135,7 +4135,7 @@
         <v>105</v>
       </c>
       <c r="K16" s="16" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -4170,7 +4170,7 @@
         <v>156</v>
       </c>
       <c r="K17" s="18" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4205,7 +4205,7 @@
         <v>156</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>106</v>
+        <v>724</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7699,7 +7699,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="34" t="s">
         <v>618</v>
       </c>
       <c r="B19" s="29"/>
@@ -7710,7 +7710,7 @@
       <c r="G19" s="29"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="34" t="s">
         <v>619</v>
       </c>
       <c r="B20" s="29"/>
@@ -7721,7 +7721,7 @@
       <c r="G20" s="29"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="34" t="s">
         <v>620</v>
       </c>
       <c r="B21" s="29"/>

</xml_diff>

<commit_message>
W3-T06 performans dogrulamasi - profile modu, Android emulatoru, Impeller/OpenGLES
- UI thread: build 0.5 ms, layout <0.1 ms, paint 0.9 ms -> 16.6 ms butcesinin
  cok altinda; Dart tarafinda darbogaz yok.
- Bosta (kontrol testi): hic kare uretilmedi, ortam gurultusu yok.
- Saf surukleme testi: cubuklarin cogunlugu butce icinde.
- Jank'in tamami RASTER asamasinda ve kart gecislerinde yogunlasti;
  sebebi gorselin GPU dokusuna ilk yuklenmesi.
- Iyilestirme: RepaintBoundary (kart surukleme boyunca yeniden rasterize
  edilmiyor) + ekran cozunurlugune bagli memCacheWidth.
- Sonuc: ortalama 57 FPS -> 88 FPS.
- Not: Emulatorde GPU yazilimla taklit edildiginden raster sureleri gercek
  cihazi temsil etmez; UI thread olcumu cihazdan bagimsiz gecerlidir.
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34CD7E68-5065-4A11-A3A9-D59F6E0F8081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D22415-7E0E-45F7-A2FE-DB33D2E6EDD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2481,6 +2481,18 @@
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -2495,25 +2507,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2927,24 +2927,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -2955,181 +2955,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="40"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3194,11 +3194,11 @@
       </c>
       <c r="D24" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$65,'Sprint Plani'!$A$4:$A$65,$A24,'Sprint Plani'!$K$4:$K$65,"Tamamlandı")</f>
-        <v>7.5</v>
+        <v>13</v>
       </c>
       <c r="E24" s="7">
         <f>IFERROR($D24/$C24,0)</f>
-        <v>0.15306122448979592</v>
+        <v>0.26530612244897961</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>43</v>
@@ -3242,11 +3242,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>43.5</v>
+        <v>49</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.3359073359073359</v>
+        <v>0.3783783783783784</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3531,85 +3531,77 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="B46" s="29"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="29"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="36" t="s">
+      <c r="A47" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="B47" s="29"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
-      <c r="F47" s="29"/>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="36" t="s">
+      <c r="A48" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="B48" s="29"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="29"/>
-      <c r="F48" s="29"/>
+      <c r="B48" s="33"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="33"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="36" t="s">
+      <c r="A49" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="B49" s="29"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="29"/>
-      <c r="E49" s="29"/>
-      <c r="F49" s="29"/>
+      <c r="B49" s="33"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="33"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="36" t="s">
+      <c r="A50" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="B50" s="29"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="29"/>
-      <c r="E50" s="29"/>
-      <c r="F50" s="29"/>
+      <c r="B50" s="33"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="33"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="33"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="36" t="s">
+      <c r="A51" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="B51" s="29"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="29"/>
-      <c r="E51" s="29"/>
-      <c r="F51" s="29"/>
+      <c r="B51" s="33"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="33"/>
+      <c r="E51" s="33"/>
+      <c r="F51" s="33"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="36" t="s">
+      <c r="A52" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="29"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="29"/>
-      <c r="E52" s="29"/>
-      <c r="F52" s="29"/>
+      <c r="B52" s="33"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="33"/>
+      <c r="E52" s="33"/>
+      <c r="F52" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3626,6 +3618,14 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3652,34 +3652,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
     </row>
     <row r="3" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -4381,26 +4381,26 @@
         <v>721</v>
       </c>
     </row>
-    <row r="23" spans="1:11" s="38" customFormat="1" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="37" t="s">
+    <row r="23" spans="1:11" s="29" customFormat="1" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="37" t="s">
+      <c r="B23" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="C23" s="28" t="s">
         <v>723</v>
       </c>
-      <c r="D23" s="37" t="s">
+      <c r="D23" s="28" t="s">
         <v>724</v>
       </c>
-      <c r="E23" s="37" t="s">
+      <c r="E23" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="F23" s="40" t="s">
+      <c r="F23" s="31" t="s">
         <v>726</v>
       </c>
-      <c r="G23" s="37" t="s">
+      <c r="G23" s="28" t="s">
         <v>727</v>
       </c>
       <c r="H23" s="18">
@@ -4448,7 +4448,7 @@
         <v>723</v>
       </c>
       <c r="K24" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -4483,7 +4483,7 @@
         <v>190</v>
       </c>
       <c r="K25" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
@@ -4518,7 +4518,7 @@
         <v>190</v>
       </c>
       <c r="K26" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5186,38 +5186,38 @@
         <v>106</v>
       </c>
     </row>
-    <row r="46" spans="1:11" s="38" customFormat="1" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="37" t="s">
+    <row r="46" spans="1:11" s="29" customFormat="1" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="37" t="s">
+      <c r="B46" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="C46" s="37" t="s">
+      <c r="C46" s="28" t="s">
         <v>287</v>
       </c>
-      <c r="D46" s="37" t="s">
+      <c r="D46" s="28" t="s">
         <v>121</v>
       </c>
-      <c r="E46" s="37" t="s">
+      <c r="E46" s="28" t="s">
         <v>728</v>
       </c>
-      <c r="F46" s="37" t="s">
+      <c r="F46" s="28" t="s">
         <v>729</v>
       </c>
-      <c r="G46" s="37" t="s">
+      <c r="G46" s="28" t="s">
         <v>730</v>
       </c>
-      <c r="H46" s="39">
+      <c r="H46" s="30">
         <v>1.5</v>
       </c>
-      <c r="I46" s="37" t="s">
+      <c r="I46" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="J46" s="37" t="s">
+      <c r="J46" s="28" t="s">
         <v>731</v>
       </c>
-      <c r="K46" s="37" t="s">
+      <c r="K46" s="28" t="s">
         <v>106</v>
       </c>
     </row>
@@ -5887,15 +5887,15 @@
       </c>
     </row>
     <row r="66" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="32" t="s">
+      <c r="A66" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="B66" s="33"/>
-      <c r="C66" s="33"/>
-      <c r="D66" s="33"/>
-      <c r="E66" s="33"/>
-      <c r="F66" s="33"/>
-      <c r="G66" s="33"/>
+      <c r="B66" s="37"/>
+      <c r="C66" s="37"/>
+      <c r="D66" s="37"/>
+      <c r="E66" s="37"/>
+      <c r="F66" s="37"/>
+      <c r="G66" s="37"/>
       <c r="H66" s="21">
         <f>SUM(H4:H65)</f>
         <v>129.5</v>
@@ -5908,64 +5908,64 @@
       <c r="K66" s="20"/>
     </row>
     <row r="68" spans="1:11" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="30" t="s">
+      <c r="A68" s="34" t="s">
         <v>376</v>
       </c>
-      <c r="B68" s="29"/>
-      <c r="C68" s="29"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="29"/>
-      <c r="F68" s="29"/>
-      <c r="G68" s="29"/>
-      <c r="H68" s="29"/>
-      <c r="I68" s="29"/>
-      <c r="J68" s="29"/>
-      <c r="K68" s="29"/>
+      <c r="B68" s="33"/>
+      <c r="C68" s="33"/>
+      <c r="D68" s="33"/>
+      <c r="E68" s="33"/>
+      <c r="F68" s="33"/>
+      <c r="G68" s="33"/>
+      <c r="H68" s="33"/>
+      <c r="I68" s="33"/>
+      <c r="J68" s="33"/>
+      <c r="K68" s="33"/>
     </row>
     <row r="69" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="30" t="s">
+      <c r="A69" s="34" t="s">
         <v>377</v>
       </c>
-      <c r="B69" s="29"/>
-      <c r="C69" s="29"/>
-      <c r="D69" s="29"/>
-      <c r="E69" s="29"/>
-      <c r="F69" s="29"/>
-      <c r="G69" s="29"/>
-      <c r="H69" s="29"/>
-      <c r="I69" s="29"/>
-      <c r="J69" s="29"/>
-      <c r="K69" s="29"/>
+      <c r="B69" s="33"/>
+      <c r="C69" s="33"/>
+      <c r="D69" s="33"/>
+      <c r="E69" s="33"/>
+      <c r="F69" s="33"/>
+      <c r="G69" s="33"/>
+      <c r="H69" s="33"/>
+      <c r="I69" s="33"/>
+      <c r="J69" s="33"/>
+      <c r="K69" s="33"/>
     </row>
     <row r="70" spans="1:11" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="30" t="s">
+      <c r="A70" s="34" t="s">
         <v>378</v>
       </c>
-      <c r="B70" s="29"/>
-      <c r="C70" s="29"/>
-      <c r="D70" s="29"/>
-      <c r="E70" s="29"/>
-      <c r="F70" s="29"/>
-      <c r="G70" s="29"/>
-      <c r="H70" s="29"/>
-      <c r="I70" s="29"/>
-      <c r="J70" s="29"/>
-      <c r="K70" s="29"/>
+      <c r="B70" s="33"/>
+      <c r="C70" s="33"/>
+      <c r="D70" s="33"/>
+      <c r="E70" s="33"/>
+      <c r="F70" s="33"/>
+      <c r="G70" s="33"/>
+      <c r="H70" s="33"/>
+      <c r="I70" s="33"/>
+      <c r="J70" s="33"/>
+      <c r="K70" s="33"/>
     </row>
     <row r="71" spans="1:11" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="34" t="s">
         <v>379</v>
       </c>
-      <c r="B71" s="29"/>
-      <c r="C71" s="29"/>
-      <c r="D71" s="29"/>
-      <c r="E71" s="29"/>
-      <c r="F71" s="29"/>
-      <c r="G71" s="29"/>
-      <c r="H71" s="29"/>
-      <c r="I71" s="29"/>
-      <c r="J71" s="29"/>
-      <c r="K71" s="29"/>
+      <c r="B71" s="33"/>
+      <c r="C71" s="33"/>
+      <c r="D71" s="33"/>
+      <c r="E71" s="33"/>
+      <c r="F71" s="33"/>
+      <c r="G71" s="33"/>
+      <c r="H71" s="33"/>
+      <c r="I71" s="33"/>
+      <c r="J71" s="33"/>
+      <c r="K71" s="33"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:K65" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -5986,7 +5986,7 @@
       <formula>"Yüksek"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K47:K65 K4:K45">
+  <conditionalFormatting sqref="K4:K45 K47:K65">
     <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"Tamamlandı"</formula>
     </cfRule>
@@ -6024,24 +6024,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>380</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>381</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -6650,26 +6650,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>478</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>479</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -7388,26 +7388,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>562</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>563</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -7767,37 +7767,37 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="38" t="s">
         <v>615</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="38" t="s">
         <v>616</v>
       </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="38" t="s">
         <v>617</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7826,22 +7826,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>618</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>619</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -8103,26 +8103,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>661</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>662</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">

</xml_diff>

<commit_message>
feat(mobile): bos durumlar icin canvas ile cizilen buyuk gorsel (W3-T08)
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D22415-7E0E-45F7-A2FE-DB33D2E6EDD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7BC5606-B111-4ED7-80D6-7C7EEF140F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2507,13 +2507,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2955,181 +2955,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3194,11 +3194,11 @@
       </c>
       <c r="D24" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$65,'Sprint Plani'!$A$4:$A$65,$A24,'Sprint Plani'!$K$4:$K$65,"Tamamlandı")</f>
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E24" s="7">
         <f>IFERROR($D24/$C24,0)</f>
-        <v>0.26530612244897961</v>
+        <v>0.40816326530612246</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>43</v>
@@ -3242,11 +3242,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.3783783783783784</v>
+        <v>0.43243243243243246</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3531,7 +3531,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="40" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="33"/>
@@ -3541,7 +3541,7 @@
       <c r="F46" s="33"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="38" t="s">
+      <c r="A47" s="40" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="33"/>
@@ -3551,7 +3551,7 @@
       <c r="F47" s="33"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="38" t="s">
+      <c r="A48" s="40" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="33"/>
@@ -3561,7 +3561,7 @@
       <c r="F48" s="33"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="38" t="s">
+      <c r="A49" s="40" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="33"/>
@@ -3571,7 +3571,7 @@
       <c r="F49" s="33"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="38" t="s">
+      <c r="A50" s="40" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="33"/>
@@ -3581,7 +3581,7 @@
       <c r="F50" s="33"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="40" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="33"/>
@@ -3591,7 +3591,7 @@
       <c r="F51" s="33"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="38" t="s">
+      <c r="A52" s="40" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="33"/>
@@ -3602,6 +3602,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3618,14 +3626,6 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4553,7 +4553,7 @@
         <v>176</v>
       </c>
       <c r="K27" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -4588,7 +4588,7 @@
         <v>204</v>
       </c>
       <c r="K28" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -4623,7 +4623,7 @@
         <v>209</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -7767,7 +7767,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="40" t="s">
         <v>615</v>
       </c>
       <c r="B19" s="33"/>
@@ -7778,7 +7778,7 @@
       <c r="G19" s="33"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="40" t="s">
         <v>616</v>
       </c>
       <c r="B20" s="33"/>
@@ -7789,7 +7789,7 @@
       <c r="G20" s="33"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="40" t="s">
         <v>617</v>
       </c>
       <c r="B21" s="33"/>

</xml_diff>

<commit_message>
feat: kalori ana ekrani ve kiler okuma/durum uclari (W3-T14, W3-T18-backend)
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7BC5606-B111-4ED7-80D6-7C7EEF140F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534B8F8C-E7E3-4485-976B-125A3D2D2D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2507,13 +2507,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2955,181 +2955,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="40"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3194,11 +3194,11 @@
       </c>
       <c r="D24" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$65,'Sprint Plani'!$A$4:$A$65,$A24,'Sprint Plani'!$K$4:$K$65,"Tamamlandı")</f>
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E24" s="7">
         <f>IFERROR($D24/$C24,0)</f>
-        <v>0.40816326530612246</v>
+        <v>0.51020408163265307</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>43</v>
@@ -3242,11 +3242,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.43243243243243246</v>
+        <v>0.47104247104247104</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3531,7 +3531,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="40" t="s">
+      <c r="A46" s="38" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="33"/>
@@ -3541,7 +3541,7 @@
       <c r="F46" s="33"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="38" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="33"/>
@@ -3551,7 +3551,7 @@
       <c r="F47" s="33"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="40" t="s">
+      <c r="A48" s="38" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="33"/>
@@ -3561,7 +3561,7 @@
       <c r="F48" s="33"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="40" t="s">
+      <c r="A49" s="38" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="33"/>
@@ -3571,7 +3571,7 @@
       <c r="F49" s="33"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="40" t="s">
+      <c r="A50" s="38" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="33"/>
@@ -3581,7 +3581,7 @@
       <c r="F50" s="33"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="40" t="s">
+      <c r="A51" s="38" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="33"/>
@@ -3591,7 +3591,7 @@
       <c r="F51" s="33"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="40" t="s">
+      <c r="A52" s="38" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="33"/>
@@ -3602,14 +3602,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3626,6 +3618,14 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4658,7 +4658,7 @@
         <v>213</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -4693,7 +4693,7 @@
         <v>176</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -7767,7 +7767,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="40" t="s">
+      <c r="A19" s="38" t="s">
         <v>615</v>
       </c>
       <c r="B19" s="33"/>
@@ -7778,7 +7778,7 @@
       <c r="G19" s="33"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="38" t="s">
         <v>616</v>
       </c>
       <c r="B20" s="33"/>
@@ -7789,7 +7789,7 @@
       <c r="G20" s="33"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="38" t="s">
         <v>617</v>
       </c>
       <c r="B21" s="33"/>

</xml_diff>

<commit_message>
feat(mobile): gorsel porsiyon secimi - kase ikonlari + avuc karsilastirmasi (W3-T17)
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534B8F8C-E7E3-4485-976B-125A3D2D2D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E3C045-5221-451C-9EE6-9297DFBB44A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="733">
   <si>
     <t>OZET DASHBOARD  |  Kalan 14 Is Gunu</t>
   </si>
@@ -2264,6 +2264,9 @@
   </si>
   <si>
     <t>W3-T02B, W3-T09</t>
+  </si>
+  <si>
+    <t>Bloke</t>
   </si>
 </sst>
 </file>
@@ -2507,13 +2510,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2955,181 +2958,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3194,11 +3197,11 @@
       </c>
       <c r="D24" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$65,'Sprint Plani'!$A$4:$A$65,$A24,'Sprint Plani'!$K$4:$K$65,"Tamamlandı")</f>
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E24" s="7">
         <f>IFERROR($D24/$C24,0)</f>
-        <v>0.51020408163265307</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>43</v>
@@ -3242,11 +3245,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.47104247104247104</v>
+        <v>0.60231660231660233</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3531,7 +3534,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="40" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="33"/>
@@ -3541,7 +3544,7 @@
       <c r="F46" s="33"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="38" t="s">
+      <c r="A47" s="40" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="33"/>
@@ -3551,7 +3554,7 @@
       <c r="F47" s="33"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="38" t="s">
+      <c r="A48" s="40" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="33"/>
@@ -3561,7 +3564,7 @@
       <c r="F48" s="33"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="38" t="s">
+      <c r="A49" s="40" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="33"/>
@@ -3571,7 +3574,7 @@
       <c r="F49" s="33"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="38" t="s">
+      <c r="A50" s="40" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="33"/>
@@ -3581,7 +3584,7 @@
       <c r="F50" s="33"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="40" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="33"/>
@@ -3591,7 +3594,7 @@
       <c r="F51" s="33"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="38" t="s">
+      <c r="A52" s="40" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="33"/>
@@ -3602,6 +3605,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3618,14 +3629,6 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4727,8 +4730,8 @@
       <c r="J32" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="K32" s="18" t="s">
-        <v>106</v>
+      <c r="K32" s="16" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -4763,7 +4766,7 @@
         <v>221</v>
       </c>
       <c r="K33" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4797,8 +4800,8 @@
       <c r="J34" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="K34" s="18" t="s">
-        <v>106</v>
+      <c r="K34" s="16" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4833,7 +4836,7 @@
         <v>176</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -4868,7 +4871,7 @@
         <v>238</v>
       </c>
       <c r="K36" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -4902,8 +4905,8 @@
       <c r="J37" s="16" t="s">
         <v>242</v>
       </c>
-      <c r="K37" s="16" t="s">
-        <v>106</v>
+      <c r="K37" s="18" t="s">
+        <v>732</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -4938,7 +4941,7 @@
         <v>246</v>
       </c>
       <c r="K38" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4973,7 +4976,7 @@
         <v>176</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -5008,7 +5011,7 @@
         <v>156</v>
       </c>
       <c r="K40" s="18" t="s">
-        <v>106</v>
+        <v>732</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -5042,8 +5045,8 @@
       <c r="J41" s="16" t="s">
         <v>260</v>
       </c>
-      <c r="K41" s="16" t="s">
-        <v>106</v>
+      <c r="K41" s="18" t="s">
+        <v>732</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5078,7 +5081,7 @@
         <v>217</v>
       </c>
       <c r="K42" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="79.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -5986,7 +5989,7 @@
       <formula>"Yüksek"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K45 K47:K65">
+  <conditionalFormatting sqref="K47:K65 K4:K45">
     <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"Tamamlandı"</formula>
     </cfRule>
@@ -5998,7 +6001,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" promptTitle="Durum" prompt="Yapılacak / Devam Ediyor / Tamamlandı / Bloke" sqref="K4:K45 K47:K65" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" promptTitle="Durum" prompt="Yapılacak / Devam Ediyor / Tamamlandı / Bloke" sqref="K47:K65 K4:K45" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Yapılacak,Devam Ediyor,Tamamlandı,Bloke"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7767,7 +7770,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="40" t="s">
         <v>615</v>
       </c>
       <c r="B19" s="33"/>
@@ -7778,7 +7781,7 @@
       <c r="G19" s="33"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="40" t="s">
         <v>616</v>
       </c>
       <c r="B20" s="33"/>
@@ -7789,7 +7792,7 @@
       <c r="G20" s="33"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="40" t="s">
         <v>617</v>
       </c>
       <c r="B21" s="33"/>

</xml_diff>

<commit_message>
feat(test): genel fotodan görme modeli doğruluk ölçümü yapan temeli yazdım
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
+++ b/docs/Kalori_Sayaci_Kalan_14_Gun_Plani.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E3C045-5221-451C-9EE6-9297DFBB44A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48099774-C326-4DE2-9E1C-C7856E30C7A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2510,13 +2510,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2958,181 +2958,181 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="40"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -3221,11 +3221,11 @@
       </c>
       <c r="D25" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$65,'Sprint Plani'!$A$4:$A$65,$A25,'Sprint Plani'!$K$4:$K$65,"Tamamlandı")</f>
-        <v>0</v>
+        <v>15.5</v>
       </c>
       <c r="E25" s="7">
         <f>IFERROR($D25/$C25,0)</f>
-        <v>0</v>
+        <v>0.34831460674157305</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>45</v>
@@ -3245,11 +3245,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D23:D25)</f>
-        <v>78</v>
+        <v>93.5</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.60231660231660233</v>
+        <v>0.72200772200772201</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -3534,7 +3534,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="40" t="s">
+      <c r="A46" s="38" t="s">
         <v>81</v>
       </c>
       <c r="B46" s="33"/>
@@ -3544,7 +3544,7 @@
       <c r="F46" s="33"/>
     </row>
     <row r="47" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="38" t="s">
         <v>82</v>
       </c>
       <c r="B47" s="33"/>
@@ -3554,7 +3554,7 @@
       <c r="F47" s="33"/>
     </row>
     <row r="48" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="40" t="s">
+      <c r="A48" s="38" t="s">
         <v>83</v>
       </c>
       <c r="B48" s="33"/>
@@ -3564,7 +3564,7 @@
       <c r="F48" s="33"/>
     </row>
     <row r="49" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="40" t="s">
+      <c r="A49" s="38" t="s">
         <v>84</v>
       </c>
       <c r="B49" s="33"/>
@@ -3574,7 +3574,7 @@
       <c r="F49" s="33"/>
     </row>
     <row r="50" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="40" t="s">
+      <c r="A50" s="38" t="s">
         <v>85</v>
       </c>
       <c r="B50" s="33"/>
@@ -3584,7 +3584,7 @@
       <c r="F50" s="33"/>
     </row>
     <row r="51" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="40" t="s">
+      <c r="A51" s="38" t="s">
         <v>86</v>
       </c>
       <c r="B51" s="33"/>
@@ -3594,7 +3594,7 @@
       <c r="F51" s="33"/>
     </row>
     <row r="52" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="40" t="s">
+      <c r="A52" s="38" t="s">
         <v>87</v>
       </c>
       <c r="B52" s="33"/>
@@ -3605,14 +3605,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A52:F52"/>
@@ -3629,6 +3621,14 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5115,8 +5115,8 @@
       <c r="J43" s="16" t="s">
         <v>255</v>
       </c>
-      <c r="K43" s="16" t="s">
-        <v>106</v>
+      <c r="K43" s="18" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
@@ -5151,7 +5151,7 @@
         <v>274</v>
       </c>
       <c r="K44" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5185,8 +5185,8 @@
       <c r="J45" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="K45" s="16" t="s">
-        <v>106</v>
+      <c r="K45" s="18" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5220,8 +5220,8 @@
       <c r="J46" s="28" t="s">
         <v>731</v>
       </c>
-      <c r="K46" s="28" t="s">
-        <v>106</v>
+      <c r="K46" s="18" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="67.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5255,8 +5255,8 @@
       <c r="J47" s="16" t="s">
         <v>255</v>
       </c>
-      <c r="K47" s="16" t="s">
-        <v>106</v>
+      <c r="K47" s="18" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -5325,8 +5325,8 @@
       <c r="J49" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="K49" s="16" t="s">
-        <v>106</v>
+      <c r="K49" s="18" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -5431,7 +5431,7 @@
         <v>288</v>
       </c>
       <c r="K52" s="18" t="s">
-        <v>106</v>
+        <v>721</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -5989,7 +5989,7 @@
       <formula>"Yüksek"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K47:K65 K4:K45">
+  <conditionalFormatting sqref="K4:K65">
     <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"Tamamlandı"</formula>
     </cfRule>
@@ -6001,7 +6001,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" promptTitle="Durum" prompt="Yapılacak / Devam Ediyor / Tamamlandı / Bloke" sqref="K47:K65 K4:K45" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" promptTitle="Durum" prompt="Yapılacak / Devam Ediyor / Tamamlandı / Bloke" sqref="K4:K65" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Yapılacak,Devam Ediyor,Tamamlandı,Bloke"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7770,7 +7770,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="40" t="s">
+      <c r="A19" s="38" t="s">
         <v>615</v>
       </c>
       <c r="B19" s="33"/>
@@ -7781,7 +7781,7 @@
       <c r="G19" s="33"/>
     </row>
     <row r="20" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="38" t="s">
         <v>616</v>
       </c>
       <c r="B20" s="33"/>
@@ -7792,7 +7792,7 @@
       <c r="G20" s="33"/>
     </row>
     <row r="21" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="38" t="s">
         <v>617</v>
       </c>
       <c r="B21" s="33"/>

</xml_diff>